<commit_message>
Reformatação lista requisitos p/ressaltar topicos
Reformatação da lista de requisitos para ressaltar topicos
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\Projetos2SI-2026\Projetos2SIPF\PastaDocsEngenhariaSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70570A6D-84D2-4DC3-99EC-7925DB570287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E042CB8-3346-4136-B044-621ACB1CB5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,9 +30,6 @@
     <t>LISTA DE REQUISITOS DO PROJETO DO SISTEMA DE GERENCIAMENTO DE ESTACIONAMENTO</t>
   </si>
   <si>
-    <t>*Legenda: Rf - Requisito funcional; Rnf - Requisito não funcional</t>
-  </si>
-  <si>
     <t>Id*</t>
   </si>
   <si>
@@ -41,12 +38,35 @@
   <si>
     <t>Descrição da regra de domínio (regra de negócio/de operação)</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">*Legenda: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rf - Requisito funcional; Rnf - Requisito não funcional</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -54,13 +74,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -90,9 +131,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -381,24 +424,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Reformatacao lista requisitos orginal recuperada
Reformatacao da lista de requisitos orginal recuperada
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\Projetos2SI-2026\Projetos2SIPF\PastaDocsEngenhariaSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E042CB8-3346-4136-B044-621ACB1CB5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF34F83-08B0-4DAD-9B34-59FB9F8C1764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48,7 +48,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">*Legenda: </t>
+      <t>*Legenda:</t>
     </r>
     <r>
       <rPr>
@@ -58,7 +58,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Rf - Requisito funcional; Rnf - Requisito não funcional</t>
+      <t xml:space="preserve"> Rf - Requisito funcional; Rnf - Requisito não funcional</t>
     </r>
   </si>
 </sst>
@@ -66,7 +66,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,8 +89,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -99,7 +107,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="-0.249977111117893"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -131,11 +145,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,18 +444,19 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="B2" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2a versao da lista com dados de pesquisas mercado
2a versao da lista de requisitos com dados de pesquisas de referencias de sistemas de mercado
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\Projetos2SI-2026\Projetos2SIPF\PastaDocsEngenhariaSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EF34F83-08B0-4DAD-9B34-59FB9F8C1764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2D5180-3594-4B0C-954D-2A242D14B098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>LISTA DE REQUISITOS DO PROJETO DO SISTEMA DE GERENCIAMENTO DE ESTACIONAMENTO</t>
   </si>
@@ -61,12 +61,138 @@
       <t xml:space="preserve"> Rf - Requisito funcional; Rnf - Requisito não funcional</t>
     </r>
   </si>
+  <si>
+    <t>Sistema deve rodar em interface WEB para PC/Note/Mobile</t>
+  </si>
+  <si>
+    <t>Rnf001</t>
+  </si>
+  <si>
+    <t>Usar linguagem de programação para aplicações WEB</t>
+  </si>
+  <si>
+    <t>Comunicar com sistemas de meio de pagamento</t>
+  </si>
+  <si>
+    <t>Usar os protocolos de interface dos meios de pagamento CIELO, REDECARD e PIX</t>
+  </si>
+  <si>
+    <t>Rf001</t>
+  </si>
+  <si>
+    <t>Emissão de nota/cupom fiscal</t>
+  </si>
+  <si>
+    <t>Integrar com impressora fiscal e sistema da Receita (Secretaria da Fazenda)</t>
+  </si>
+  <si>
+    <t>Rf002</t>
+  </si>
+  <si>
+    <t>Suporte para conveniados</t>
+  </si>
+  <si>
+    <t>Tabela de preços específica para convênios com empresas</t>
+  </si>
+  <si>
+    <t>Rf003</t>
+  </si>
+  <si>
+    <t>Rnf002</t>
+  </si>
+  <si>
+    <t>Padrão das telas do sistema</t>
+  </si>
+  <si>
+    <t>Fundo azul marinho com letras em branco, logo da empresa usuária do sistema no topo da tela do lado direito</t>
+  </si>
+  <si>
+    <t>Dashboard de consulta de quantidade média de veículos por dia da semana</t>
+  </si>
+  <si>
+    <t>Dashboard do dia de pico de cada mês no último ano</t>
+  </si>
+  <si>
+    <t>Dashboard de valor faturado por dia/mês no último ano</t>
+  </si>
+  <si>
+    <t>Rnf003</t>
+  </si>
+  <si>
+    <t>Os dashboards gerenciais precisam ficar na mesma tela</t>
+  </si>
+  <si>
+    <t>Rf004</t>
+  </si>
+  <si>
+    <t>Rf005</t>
+  </si>
+  <si>
+    <t>Rf006</t>
+  </si>
+  <si>
+    <t>Criar áreas separadas em janelas na tela de consulta</t>
+  </si>
+  <si>
+    <t>Mostrar um gráfico de barras com as datas no eixo X e quantidades no eixo Y</t>
+  </si>
+  <si>
+    <t>Mostrar um relatório em forma de tabela com os dias de pico de cada mês e a quantidade de carros movimentada no dia</t>
+  </si>
+  <si>
+    <t>Mostrar um gráfico de linhas com as datas no eixo X e os valores faturados no eixo Y</t>
+  </si>
+  <si>
+    <t>Notificação de proximidade do horário de fechamento</t>
+  </si>
+  <si>
+    <t>Avisar por Whatsapp que o estacionamento vai fechar, com 1 mensagem aos 30 min antes, 1 aos 10 min antes</t>
+  </si>
+  <si>
+    <t>Rf007</t>
+  </si>
+  <si>
+    <t>Notificação do tempo de permanência</t>
+  </si>
+  <si>
+    <t>A cada 30 min estacionado, enviar aviso por Whatsapp ao cliente com o tempo e o valor do momento</t>
+  </si>
+  <si>
+    <t>Rf008</t>
+  </si>
+  <si>
+    <t>Controle de status de ocupação de vagas</t>
+  </si>
+  <si>
+    <t>Cada vaga tem status de ocupada ou livre</t>
+  </si>
+  <si>
+    <t>Rf009</t>
+  </si>
+  <si>
+    <t>Leitura automática de placas</t>
+  </si>
+  <si>
+    <t>Vincular cadastro de veículo com placa, agilizando a entrada e saída</t>
+  </si>
+  <si>
+    <t>Rf010</t>
+  </si>
+  <si>
+    <t>Rf011</t>
+  </si>
+  <si>
+    <t>Suporte para redes de estacionamentos</t>
+  </si>
+  <si>
+    <t>Permitir controlar mais de um estacionamento, suas vagas e movimentos</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -93,6 +219,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -431,10 +563,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="50.7109375" customWidth="1"/>
+    <col min="2" max="2" width="54.42578125" customWidth="1"/>
     <col min="3" max="3" width="126.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -461,19 +593,37 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
@@ -481,76 +631,349 @@
       <c r="C8" s="1"/>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+      <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="A12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="A13" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="A14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="A15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="A16" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="A17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="A18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
+      <c r="A19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007544514C3E525041A50FD90CCA057415" ma:contentTypeVersion="10" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="bf4730f3f1a762055629886e8f42d477">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b591360b-72bd-45d7-9362-d2d404a7b4f5" xmlns:ns3="e265a0ad-4171-4359-86dd-7b4a7d920c0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e150f1db5eef3c20961c9854c2263c4" ns2:_="" ns3:_="">
+    <xsd:import namespace="b591360b-72bd-45d7-9362-d2d404a7b4f5"/>
+    <xsd:import namespace="e265a0ad-4171-4359-86dd-7b4a7d920c0e"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b591360b-72bd-45d7-9362-d2d404a7b4f5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e2398b20-2c76-408b-9565-673d41e5947a" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="e265a0ad-4171-4359-86dd-7b4a7d920c0e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{8c11a7f7-aad1-42b2-b41d-2cd932099fb5}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="e265a0ad-4171-4359-86dd-7b4a7d920c0e">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e265a0ad-4171-4359-86dd-7b4a7d920c0e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800DB960-F05E-4141-AFC3-FD43E9D5A7C9}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D1F747B-A076-4329-9D35-44DBCC6CEFE3}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07439A18-58BE-4AE4-8428-3F424A8958CB}"/>
 </file>
</xml_diff>

<commit_message>
3a versao da lista com Brainstorm
</commit_message>
<xml_diff>
--- a/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
+++ b/PastaDocsEngenhariaSw/ListaRequisitosSiEstacionamento.xlsx
@@ -1,42 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29930"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\Projetos2SI-2026\Projetos2SIPF\PastaDocsEngenhariaSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2D5180-3594-4B0C-954D-2A242D14B098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{1C2D5180-3594-4B0C-954D-2A242D14B098}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7959D08E-FB2B-490C-8512-4035941AF628}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>LISTA DE REQUISITOS DO PROJETO DO SISTEMA DE GERENCIAMENTO DE ESTACIONAMENTO</t>
-  </si>
-  <si>
-    <t>Id*</t>
-  </si>
-  <si>
-    <t>Nome do requisito</t>
-  </si>
-  <si>
-    <t>Descrição da regra de domínio (regra de negócio/de operação)</t>
   </si>
   <si>
     <r>
@@ -62,22 +64,70 @@
     </r>
   </si>
   <si>
+    <t>Id*</t>
+  </si>
+  <si>
+    <t>Nome do requisito</t>
+  </si>
+  <si>
+    <t>Descrição da regra de domínio (regra de negócio/de operação)</t>
+  </si>
+  <si>
+    <t>Rnf001</t>
+  </si>
+  <si>
     <t>Sistema deve rodar em interface WEB para PC/Note/Mobile</t>
   </si>
   <si>
-    <t>Rnf001</t>
-  </si>
-  <si>
     <t>Usar linguagem de programação para aplicações WEB</t>
   </si>
   <si>
+    <t>Rnf002</t>
+  </si>
+  <si>
+    <t>Padrão das telas do sistema</t>
+  </si>
+  <si>
+    <t>Fundo azul marinho com letras em branco, logo da empresa usuária do sistema no topo da tela do lado direito</t>
+  </si>
+  <si>
+    <t>Rnf003</t>
+  </si>
+  <si>
+    <t>Os dashboards gerenciais precisam ficar na mesma tela</t>
+  </si>
+  <si>
+    <t>Criar áreas separadas em janelas na tela de consulta</t>
+  </si>
+  <si>
+    <t>Rnf004</t>
+  </si>
+  <si>
+    <t>Disponibilidade Offline</t>
+  </si>
+  <si>
+    <t>O sistema deve operar localmente em caso de queda de link de internet</t>
+  </si>
+  <si>
+    <t>Rnf005</t>
+  </si>
+  <si>
+    <t>Conformidade LGPD</t>
+  </si>
+  <si>
+    <t>Criptografia de dados pessoais e opção de anonimização de histórico</t>
+  </si>
+  <si>
+    <t>Rf001</t>
+  </si>
+  <si>
     <t>Comunicar com sistemas de meio de pagamento</t>
   </si>
   <si>
     <t>Usar os protocolos de interface dos meios de pagamento CIELO, REDECARD e PIX</t>
   </si>
   <si>
-    <t>Rf001</t>
+    <t>Rf002</t>
   </si>
   <si>
     <t>Emissão de nota/cupom fiscal</t>
@@ -86,7 +136,7 @@
     <t>Integrar com impressora fiscal e sistema da Receita (Secretaria da Fazenda)</t>
   </si>
   <si>
-    <t>Rf002</t>
+    <t>Rf003</t>
   </si>
   <si>
     <t>Suporte para conveniados</t>
@@ -95,61 +145,43 @@
     <t>Tabela de preços específica para convênios com empresas</t>
   </si>
   <si>
-    <t>Rf003</t>
-  </si>
-  <si>
-    <t>Rnf002</t>
-  </si>
-  <si>
-    <t>Padrão das telas do sistema</t>
-  </si>
-  <si>
-    <t>Fundo azul marinho com letras em branco, logo da empresa usuária do sistema no topo da tela do lado direito</t>
+    <t>Rf004</t>
   </si>
   <si>
     <t>Dashboard de consulta de quantidade média de veículos por dia da semana</t>
   </si>
   <si>
+    <t>Mostrar um gráfico de barras com as datas no eixo X e quantidades no eixo Y</t>
+  </si>
+  <si>
+    <t>Rf005</t>
+  </si>
+  <si>
     <t>Dashboard do dia de pico de cada mês no último ano</t>
   </si>
   <si>
+    <t>Mostrar um relatório em forma de tabela com os dias de pico de cada mês e a quantidade de carros movimentada no dia</t>
+  </si>
+  <si>
+    <t>Rf006</t>
+  </si>
+  <si>
     <t>Dashboard de valor faturado por dia/mês no último ano</t>
   </si>
   <si>
-    <t>Rnf003</t>
-  </si>
-  <si>
-    <t>Os dashboards gerenciais precisam ficar na mesma tela</t>
-  </si>
-  <si>
-    <t>Rf004</t>
-  </si>
-  <si>
-    <t>Rf005</t>
-  </si>
-  <si>
-    <t>Rf006</t>
-  </si>
-  <si>
-    <t>Criar áreas separadas em janelas na tela de consulta</t>
-  </si>
-  <si>
-    <t>Mostrar um gráfico de barras com as datas no eixo X e quantidades no eixo Y</t>
-  </si>
-  <si>
-    <t>Mostrar um relatório em forma de tabela com os dias de pico de cada mês e a quantidade de carros movimentada no dia</t>
-  </si>
-  <si>
     <t>Mostrar um gráfico de linhas com as datas no eixo X e os valores faturados no eixo Y</t>
   </si>
   <si>
+    <t>Rf007</t>
+  </si>
+  <si>
     <t>Notificação de proximidade do horário de fechamento</t>
   </si>
   <si>
     <t>Avisar por Whatsapp que o estacionamento vai fechar, com 1 mensagem aos 30 min antes, 1 aos 10 min antes</t>
   </si>
   <si>
-    <t>Rf007</t>
+    <t>Rf008</t>
   </si>
   <si>
     <t>Notificação do tempo de permanência</t>
@@ -158,7 +190,7 @@
     <t>A cada 30 min estacionado, enviar aviso por Whatsapp ao cliente com o tempo e o valor do momento</t>
   </si>
   <si>
-    <t>Rf008</t>
+    <t>Rf009</t>
   </si>
   <si>
     <t>Controle de status de ocupação de vagas</t>
@@ -167,7 +199,7 @@
     <t>Cada vaga tem status de ocupada ou livre</t>
   </si>
   <si>
-    <t>Rf009</t>
+    <t>Rf010</t>
   </si>
   <si>
     <t>Leitura automática de placas</t>
@@ -176,9 +208,6 @@
     <t>Vincular cadastro de veículo com placa, agilizando a entrada e saída</t>
   </si>
   <si>
-    <t>Rf010</t>
-  </si>
-  <si>
     <t>Rf011</t>
   </si>
   <si>
@@ -186,13 +215,91 @@
   </si>
   <si>
     <t>Permitir controlar mais de um estacionamento, suas vagas e movimentos</t>
+  </si>
+  <si>
+    <t>Rf012</t>
+  </si>
+  <si>
+    <t>Gestão de pagamento de Mensalistas</t>
+  </si>
+  <si>
+    <t>Controle de pagamentos com boleto, PIX ou Cartão e vencimentos</t>
+  </si>
+  <si>
+    <t>Rf013</t>
+  </si>
+  <si>
+    <t>Gestão de pagamento de avulsos</t>
+  </si>
+  <si>
+    <t>Controle de pagamentos com tabel de preços por dia/horário/permanência</t>
+  </si>
+  <si>
+    <t>Rd014</t>
+  </si>
+  <si>
+    <t>Gestão de Controle de Caixa</t>
+  </si>
+  <si>
+    <t>Exigir rotina de abertura e fechamento de caixa por cada usuario, registrando valor inicial e final do caixa.</t>
+  </si>
+  <si>
+    <t>Rf015</t>
+  </si>
+  <si>
+    <t>Medidas de segurança</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impedimento de fraudes por meio de registros com fotos e códigos </t>
+  </si>
+  <si>
+    <t>Rf016</t>
+  </si>
+  <si>
+    <t>Controle de vagas para carros eletricos</t>
+  </si>
+  <si>
+    <t>Mostrar quais vagas do estacionamento sao especificas para carros eletricos com carregador para poder usar</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>Rf017</t>
+  </si>
+  <si>
+    <t>Bloqueio de mensalistas e conveniados por falta de pagamento</t>
+  </si>
+  <si>
+    <t>Após 15 das em atraso de mensalidade, bloquear a entrada (emitir aviso ao operador da recepção ou bloquear cancela)</t>
+  </si>
+  <si>
+    <t>e/</t>
+  </si>
+  <si>
+    <t>Rf018</t>
+  </si>
+  <si>
+    <t>Registro de Avarias</t>
+  </si>
+  <si>
+    <t>Registrar fotos do veículo na entrada para evitar falsas queixas de danos</t>
+  </si>
+  <si>
+    <t>Rf019</t>
+  </si>
+  <si>
+    <t>Vagas EV de prioridade e compatibilidade</t>
+  </si>
+  <si>
+    <t>Apenas veículos com permissão podem ocupar vagas marcadas com EV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -563,193 +670,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="54.42578125" customWidth="1"/>
     <col min="3" max="3" width="126.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" customFormat="1">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" customFormat="1">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="1" t="s">
+    <row r="10" spans="1:3" customFormat="1">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="1:3" customFormat="1">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:3" customFormat="1">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:3" customFormat="1">
+      <c r="A13" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" customFormat="1">
+      <c r="A14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" customFormat="1">
+      <c r="A15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" customFormat="1">
+      <c r="A16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+    <row r="17" spans="1:4">
+      <c r="A17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>46</v>
       </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="17.25" customHeight="1">
+      <c r="A24" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D28" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D29" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -758,6 +1016,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="e265a0ad-4171-4359-86dd-7b4a7d920c0e" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007544514C3E525041A50FD90CCA057415" ma:contentTypeVersion="10" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="bf4730f3f1a762055629886e8f42d477">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b591360b-72bd-45d7-9362-d2d404a7b4f5" xmlns:ns3="e265a0ad-4171-4359-86dd-7b4a7d920c0e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e150f1db5eef3c20961c9854c2263c4" ns2:_="" ns3:_="">
     <xsd:import namespace="b591360b-72bd-45d7-9362-d2d404a7b4f5"/>
@@ -946,34 +1224,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="e265a0ad-4171-4359-86dd-7b4a7d920c0e" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b591360b-72bd-45d7-9362-d2d404a7b4f5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800DB960-F05E-4141-AFC3-FD43E9D5A7C9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D1F747B-A076-4329-9D35-44DBCC6CEFE3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3D1F747B-A076-4329-9D35-44DBCC6CEFE3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07439A18-58BE-4AE4-8428-3F424A8958CB}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07439A18-58BE-4AE4-8428-3F424A8958CB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800DB960-F05E-4141-AFC3-FD43E9D5A7C9}"/>
 </file>
</xml_diff>